<commit_message>
Ajutes Transcription > Video ID
</commit_message>
<xml_diff>
--- a/XLS/SCRAPE_single_video.xlsx
+++ b/XLS/SCRAPE_single_video.xlsx
@@ -427,30 +427,30 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Animais da Amazônia Que Podem Desaparecer!😱
-#animais #natureza #curiosidades #a</v>
+        <v xml:space="preserve">O Homem Invisível do Rio Finalmente Caiu
+#creatorsearchinsights #noticiastiktok </v>
       </c>
       <c r="B2">
-        <v>593500</v>
+        <v>132400</v>
       </c>
       <c r="C2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Animais da Amazônia Que Podem Desaparecer!😱
-#animais #natureza #curiosidades #animals </v>
+        <v xml:space="preserve">O Homem Invisível do Rio Finalmente Caiu
+#creatorsearchinsights #noticiastiktok #noticia #jornalismo #crimeorganizado</v>
       </c>
       <c r="D2">
-        <v>21600</v>
+        <v>5769</v>
       </c>
       <c r="E2" t="str">
-        <v>animais, natureza, curiosidades, animals</v>
+        <v>creatorsearchinsights, noticiastiktok, noticia, jornalismo, crimeorganizado</v>
       </c>
       <c r="F2" t="str">
-        <v>https://www.tiktok.com/@dna.selvagem1/video/7577804139195829511</v>
+        <v>https://www.tiktok.com/@sociedadecartoon/video/7611716468035603732</v>
       </c>
       <c r="G2">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="H2" t="str">
-        <v>2025-11-28T15:50:21.000Z</v>
+        <v>2026-02-28T01:07:34.000Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Skip itens ja processados
</commit_message>
<xml_diff>
--- a/XLS/SCRAPE_single_video.xlsx
+++ b/XLS/SCRAPE_single_video.xlsx
@@ -425,32 +425,30 @@
         <v>publish_date</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>Vídeo #11 - Quer conhecer os detalhes viscerais dessa história? O livro "Heliogá</v>
+        <v/>
       </c>
       <c r="B2">
-        <v>30100</v>
-      </c>
-      <c r="C2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Vídeo #11 - Quer conhecer os detalhes viscerais dessa história? O livro "Heliogábalo: O Anarquista Coroado" está no link da bio. Acesse o perfil e procure pelo #11.
-Aconteceu exatamente no dia de hoje, 11 de março de 222 d.C. O imperador mais bizarro de Roma encontrou seu fim no esgoto da cidade. Heliogábalo zombou das tradições, sufocou a elite e testou os limites da loucura. Roma não perdoou.
-#historia #imperioromano #heliogabalo #oladocinza #curiosidadeshistoricas #romaantiga #estrategia #bizarro</v>
+        <v>205600</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
       </c>
       <c r="D2">
-        <v>1608</v>
+        <v>2961</v>
       </c>
       <c r="E2" t="str">
-        <v>historia, heliogabalo, oladocinza, curiosidadeshistoricas, romaantiga, estrategia, bizarro</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>https://www.tiktok.com/@ladocinza/video/7615831620825648385</v>
+        <v>https://www.tiktok.com/@789534ra/video/7608357297735191829</v>
       </c>
       <c r="G2">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-03-11T20:00:00.000Z</v>
+        <v>2026-02-18T23:52:24.000Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>